<commit_message>
further information in progress.txx
</commit_message>
<xml_diff>
--- a/src/accounting/exercise-hrd.xlsx
+++ b/src/accounting/exercise-hrd.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software-Developer-JS\project-accounting-electron\src\accounting\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software-Developer-JS\electron-sqlite3\src\accounting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C8F6BB-D212-4F2B-B83A-C4EAEE874748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6674AA5D-B0DF-4371-96AB-5D97327C5645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="480" windowWidth="13488" windowHeight="11976" firstSheet="2" activeTab="3" xr2:uid="{19176008-2B21-4C25-B606-0A07DF05EBBC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{19176008-2B21-4C25-B606-0A07DF05EBBC}"/>
   </bookViews>
   <sheets>
     <sheet name="exercise" sheetId="2" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <pivotCache cacheId="0" r:id="rId6"/>
     <pivotCache cacheId="1" r:id="rId7"/>
     <pivotCache cacheId="2" r:id="rId8"/>
+    <pivotCache cacheId="6" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="244">
   <si>
     <t>Date</t>
   </si>
@@ -636,9 +637,6 @@
     <t>Customer Ferdiansyah Membeli Product A dengan harga 13 juta sebanyak 5 secara tunai, penjualan ini dilakukan oleh  Salesman bernama  Wpu</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer bernama Warrent Buffet Membeli Product B dengan harga 14 juta sebanyak 10 items secara kredit dengan DP 5 juta dan bunga 10%, penjualan ini dilakukan oleh Salesman bernama Doddy </t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -775,6 +773,9 @@
   </si>
   <si>
     <t>PinemBreBirink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer bernama Warrent Buffet Membeli Product B dengan harga 14 juta sebanyak 10 items secara kredit bunga 10% lalu DP 5 juta dan, penjualan ini dilakukan oleh Salesman bernama Doddy </t>
   </si>
 </sst>
 </file>
@@ -960,7 +961,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1093,6 +1094,7 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1114,12 +1116,6 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1129,6 +1125,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1570,6 +1570,37 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="ASUS" refreshedDate="45771.060608680556" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{D0FCFA8F-460B-41CF-B94E-E01BCDCDBF3B}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="E1:H11" sheet="sale"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="ProductName" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Product A"/>
+        <s v="Product C"/>
+        <s v="Product B"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="ProductPriceSell" numFmtId="44">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="13000000" maxValue="16000000"/>
+    </cacheField>
+    <cacheField name="SaleQty" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="-1" maxValue="10"/>
+    </cacheField>
+    <cacheField name="SaleBalance" numFmtId="44">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="-13000000" maxValue="140000000"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="76">
   <r>
@@ -2489,6 +2520,71 @@
     <x v="2"/>
     <n v="2"/>
     <m/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="10"/>
+    <n v="130000000"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="5"/>
+    <n v="65000000"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="16000000"/>
+    <n v="5"/>
+    <n v="80000000"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="14000000"/>
+    <n v="5"/>
+    <n v="70000000"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="-1"/>
+    <n v="-13000000"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="5"/>
+    <n v="65000000"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="16000000"/>
+    <n v="5"/>
+    <n v="80000000"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="14000000"/>
+    <n v="10"/>
+    <n v="140000000"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="5"/>
+    <n v="65000000"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="13000000"/>
+    <n v="5"/>
+    <n v="65000000"/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -2665,6 +2761,66 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B95AB8F1-F2A9-4521-9391-8B4BDDC937A5}" name="PivotTable2" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="M7:O11" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="44" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="44" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of SaleQty" fld="2" baseField="0" baseItem="0"/>
+    <dataField name="Sum of SaleBalance" fld="3" baseField="0" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C3687B6E-F10B-4DB4-BDCF-B709FDAEEFE6}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="M1:O4" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
@@ -3223,7 +3379,7 @@
         <v>0.62777777777777777</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>197</v>
+        <v>243</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>126</v>
@@ -5506,16 +5662,16 @@
         <v>124</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K1" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="L1" s="18" t="s">
-        <v>224</v>
-      </c>
       <c r="M1" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -5661,10 +5817,10 @@
       <c r="J5" s="17">
         <v>2</v>
       </c>
-      <c r="K5" s="58" t="s">
-        <v>198</v>
-      </c>
-      <c r="L5" s="58"/>
+      <c r="K5" s="59" t="s">
+        <v>197</v>
+      </c>
+      <c r="L5" s="59"/>
       <c r="M5" s="18">
         <f>SUM(M2:M4)</f>
         <v>30000000</v>
@@ -6101,38 +6257,38 @@
       <c r="L1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="60" t="s">
+      <c r="M1" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="61"/>
+      <c r="N1" s="62"/>
       <c r="O1" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="P1" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="R1" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="R1" s="17" t="s">
-        <v>206</v>
-      </c>
       <c r="S1" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="T1" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="T1" s="18" t="s">
-        <v>205</v>
-      </c>
       <c r="U1" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="W1" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="X1" s="58"/>
-      <c r="Y1" s="58"/>
-      <c r="AA1" s="62" t="s">
-        <v>220</v>
-      </c>
-      <c r="AB1" s="63"/>
-      <c r="AC1" s="64"/>
+        <v>208</v>
+      </c>
+      <c r="W1" s="59" t="s">
+        <v>214</v>
+      </c>
+      <c r="X1" s="59"/>
+      <c r="Y1" s="59"/>
+      <c r="AA1" s="63" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB1" s="64"/>
+      <c r="AC1" s="65"/>
     </row>
     <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="28">
@@ -6188,22 +6344,22 @@
         <v>109295000</v>
       </c>
       <c r="W2" s="26" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="X2" s="31" t="s">
+        <v>203</v>
+      </c>
+      <c r="Y2" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="Y2" s="31" t="s">
+      <c r="AA2" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="AA2" s="17" t="s">
-        <v>206</v>
-      </c>
       <c r="AB2" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="AC2" s="18" t="s">
         <v>204</v>
-      </c>
-      <c r="AC2" s="18" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.3">
@@ -6319,7 +6475,7 @@
         <v>0</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="S4" s="31">
         <v>50000000</v>
@@ -6407,7 +6563,7 @@
         <v>35000000</v>
       </c>
       <c r="W5" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="X5" s="18">
         <f>U4</f>
@@ -6492,7 +6648,7 @@
         <v>35000000</v>
       </c>
       <c r="AA6" s="18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AB6" s="18">
         <f>Y14</f>
@@ -6568,7 +6724,7 @@
         <v>240000000</v>
       </c>
       <c r="AA7" s="40" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB7" s="18">
         <v>0</v>
@@ -6620,7 +6776,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S8" s="31">
         <v>13000000</v>
@@ -6700,7 +6856,7 @@
         <v>735000000</v>
       </c>
       <c r="W9" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="X9" s="18">
         <f>U8</f>
@@ -6711,7 +6867,7 @@
       </c>
       <c r="Z9" s="1"/>
       <c r="AA9" s="18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB9" s="18">
         <f>SUM(AC10:AC12)</f>
@@ -6784,7 +6940,7 @@
       </c>
       <c r="Z10" s="1"/>
       <c r="AA10" s="40" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AB10" s="18">
         <v>0</v>
@@ -6987,7 +7143,7 @@
         <v>3000000</v>
       </c>
       <c r="R13" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="S13" s="18">
         <v>0</v>
@@ -7056,7 +7212,7 @@
         <v>0</v>
       </c>
       <c r="W14" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="X14" s="18">
         <v>0</v>
@@ -7067,7 +7223,7 @@
       </c>
       <c r="Z14" s="1"/>
       <c r="AA14" s="18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB14" s="41">
         <v>30000000</v>
@@ -7119,7 +7275,7 @@
         <v>75000000</v>
       </c>
       <c r="W15" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="X15" s="18">
         <f>SUM(X3:X14)</f>
@@ -7130,7 +7286,7 @@
         <v>1069000000</v>
       </c>
       <c r="AA15" s="42" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AB15" s="18">
         <v>0</v>
@@ -7210,13 +7366,13 @@
       <c r="P17" s="31">
         <v>0</v>
       </c>
-      <c r="W17" s="69" t="s">
-        <v>232</v>
-      </c>
-      <c r="X17" s="70"/>
-      <c r="Y17" s="71"/>
+      <c r="W17" s="66" t="s">
+        <v>231</v>
+      </c>
+      <c r="X17" s="67"/>
+      <c r="Y17" s="68"/>
       <c r="AA17" s="43" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB17" s="18">
         <f>AC18</f>
@@ -7264,7 +7420,7 @@
       <c r="W18" s="46" t="s">
         <v>191</v>
       </c>
-      <c r="X18" s="67">
+      <c r="X18" s="1">
         <f>Y8</f>
         <v>760000000</v>
       </c>
@@ -7316,9 +7472,9 @@
         <v>0</v>
       </c>
       <c r="W19" s="46" t="s">
-        <v>208</v>
-      </c>
-      <c r="X19" s="67">
+        <v>207</v>
+      </c>
+      <c r="X19" s="1">
         <f>X9</f>
         <v>13000000</v>
       </c>
@@ -7360,17 +7516,17 @@
         <v>13000000</v>
       </c>
       <c r="W20" s="46" t="s">
-        <v>216</v>
-      </c>
-      <c r="X20" s="67">
+        <v>215</v>
+      </c>
+      <c r="X20" s="1">
         <v>0</v>
       </c>
       <c r="Y20" s="47"/>
-      <c r="AA20" s="65" t="s">
-        <v>239</v>
-      </c>
-      <c r="AB20" s="65"/>
-      <c r="AC20" s="65"/>
+      <c r="AA20" s="69" t="s">
+        <v>238</v>
+      </c>
+      <c r="AB20" s="69"/>
+      <c r="AC20" s="69"/>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A21" s="28">
@@ -7408,16 +7564,15 @@
         <v>0</v>
       </c>
       <c r="W21" s="46"/>
-      <c r="X21" s="67"/>
       <c r="Y21" s="47"/>
       <c r="AA21" s="43" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AB21" s="31" t="s">
+        <v>203</v>
+      </c>
+      <c r="AC21" s="31" t="s">
         <v>204</v>
-      </c>
-      <c r="AC21" s="31" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.3">
@@ -7456,9 +7611,8 @@
         <v>60000000</v>
       </c>
       <c r="W22" s="46" t="s">
-        <v>217</v>
-      </c>
-      <c r="X22" s="67"/>
+        <v>216</v>
+      </c>
       <c r="Y22" s="50">
         <f>X18-X19-X20</f>
         <v>747000000</v>
@@ -7512,7 +7666,6 @@
         <v>0</v>
       </c>
       <c r="W23" s="46"/>
-      <c r="X23" s="67"/>
       <c r="Y23" s="47"/>
       <c r="AA23" s="18" t="str">
         <f t="shared" si="0"/>
@@ -7563,9 +7716,9 @@
         <v>0</v>
       </c>
       <c r="W24" s="46" t="s">
-        <v>218</v>
-      </c>
-      <c r="X24" s="67">
+        <v>217</v>
+      </c>
+      <c r="X24" s="1">
         <f>X10</f>
         <v>735000000</v>
       </c>
@@ -7621,7 +7774,7 @@
       <c r="W25" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="X25" s="67">
+      <c r="X25" s="1">
         <f>Y11</f>
         <v>12000000</v>
       </c>
@@ -7674,7 +7827,7 @@
       <c r="W26" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="X26" s="67">
+      <c r="X26" s="1">
         <f>Y12</f>
         <v>3000000</v>
       </c>
@@ -7725,9 +7878,9 @@
         <v>1500000</v>
       </c>
       <c r="W27" s="46" t="s">
-        <v>221</v>
-      </c>
-      <c r="X27" s="67">
+        <v>220</v>
+      </c>
+      <c r="X27" s="1">
         <f>X24-X25-X26</f>
         <v>720000000</v>
       </c>
@@ -7778,14 +7931,14 @@
         <v>3000000</v>
       </c>
       <c r="W28" s="46" t="s">
-        <v>222</v>
-      </c>
-      <c r="X28" s="67">
+        <v>221</v>
+      </c>
+      <c r="X28" s="1">
         <v>30000000</v>
       </c>
       <c r="Y28" s="47"/>
       <c r="AA28" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AB28" s="18">
         <f>SUM(AB22:AB27)</f>
@@ -7829,7 +7982,6 @@
         <v>50000000</v>
       </c>
       <c r="W29" s="46"/>
-      <c r="X29" s="67"/>
       <c r="Y29" s="47"/>
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.3">
@@ -7865,19 +8017,18 @@
         <v>0</v>
       </c>
       <c r="W30" s="46" t="s">
-        <v>225</v>
-      </c>
-      <c r="X30" s="67"/>
+        <v>224</v>
+      </c>
       <c r="Y30" s="47">
         <f>X27-X28</f>
         <v>690000000</v>
       </c>
       <c r="Z30" s="1"/>
-      <c r="AA30" s="65" t="s">
-        <v>233</v>
-      </c>
-      <c r="AB30" s="65"/>
-      <c r="AC30" s="65"/>
+      <c r="AA30" s="69" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB30" s="69"/>
+      <c r="AC30" s="69"/>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A31" s="28">
@@ -7915,10 +8066,9 @@
         <v>130000000</v>
       </c>
       <c r="W31" s="46"/>
-      <c r="X31" s="67"/>
       <c r="Y31" s="47"/>
       <c r="AA31" s="54" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AB31" s="44"/>
       <c r="AC31" s="45"/>
@@ -7959,9 +8109,8 @@
         <v>0</v>
       </c>
       <c r="W32" s="46" t="s">
-        <v>226</v>
-      </c>
-      <c r="X32" s="67"/>
+        <v>225</v>
+      </c>
       <c r="Y32" s="47">
         <f>Y22-Y30</f>
         <v>57000000</v>
@@ -8009,7 +8158,6 @@
         <v>0</v>
       </c>
       <c r="W33" s="46"/>
-      <c r="X33" s="67"/>
       <c r="Y33" s="47"/>
       <c r="AA33" s="53" t="str">
         <f>D50</f>
@@ -8057,12 +8205,11 @@
         <v>0</v>
       </c>
       <c r="W34" s="46" t="s">
-        <v>227</v>
-      </c>
-      <c r="X34" s="67"/>
+        <v>226</v>
+      </c>
       <c r="Y34" s="47"/>
       <c r="AA34" s="51" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AC34" s="47">
         <f>AB32+AB33</f>
@@ -8105,9 +8252,8 @@
         <v>120000000</v>
       </c>
       <c r="W35" s="52" t="s">
-        <v>228</v>
-      </c>
-      <c r="X35" s="67"/>
+        <v>227</v>
+      </c>
       <c r="Y35" s="47">
         <f>X13</f>
         <v>17705000</v>
@@ -8151,10 +8297,9 @@
         <v>0</v>
       </c>
       <c r="W36" s="46"/>
-      <c r="X36" s="67"/>
       <c r="Y36" s="47"/>
       <c r="AA36" s="51" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AC36" s="47"/>
     </row>
@@ -8178,9 +8323,8 @@
         <v>156</v>
       </c>
       <c r="W37" s="46" t="s">
-        <v>229</v>
-      </c>
-      <c r="X37" s="67"/>
+        <v>228</v>
+      </c>
       <c r="Y37" s="47"/>
       <c r="AA37" s="56" t="str">
         <f>D48</f>
@@ -8227,15 +8371,14 @@
         <v>0</v>
       </c>
       <c r="W38" s="53" t="s">
-        <v>230</v>
-      </c>
-      <c r="X38" s="67"/>
+        <v>229</v>
+      </c>
       <c r="Y38" s="47">
         <f>Y14</f>
         <v>19000000</v>
       </c>
       <c r="AA38" s="51" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AC38" s="47">
         <f>AC37</f>
@@ -8275,7 +8418,6 @@
         <v>0</v>
       </c>
       <c r="W39" s="46"/>
-      <c r="X39" s="67"/>
       <c r="Y39" s="47"/>
       <c r="AA39" s="51"/>
       <c r="AC39" s="47"/>
@@ -8313,15 +8455,14 @@
         <v>5000000</v>
       </c>
       <c r="W40" s="46" t="s">
-        <v>231</v>
-      </c>
-      <c r="X40" s="67"/>
+        <v>230</v>
+      </c>
       <c r="Y40" s="47">
         <f>Y32-Y35+Y38</f>
         <v>58295000</v>
       </c>
       <c r="AA40" s="51" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AC40" s="47">
         <f>AB17</f>
@@ -8348,10 +8489,9 @@
       <c r="L41" s="28"/>
       <c r="M41" s="28"/>
       <c r="N41" s="28"/>
-      <c r="W41" s="66" t="s">
-        <v>240</v>
-      </c>
-      <c r="X41" s="67"/>
+      <c r="W41" s="46" t="s">
+        <v>239</v>
+      </c>
       <c r="Y41" s="47"/>
       <c r="AA41" s="51"/>
       <c r="AC41" s="47"/>
@@ -8393,16 +8533,15 @@
       <c r="P42" s="31">
         <v>0</v>
       </c>
-      <c r="W42" s="66" t="s">
-        <v>241</v>
-      </c>
-      <c r="X42" s="67"/>
+      <c r="W42" s="46" t="s">
+        <v>240</v>
+      </c>
       <c r="Y42" s="47">
         <f>Y40*21/100</f>
         <v>12241950</v>
       </c>
       <c r="AA42" s="57" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AB42" s="48"/>
       <c r="AC42" s="49">
@@ -8434,7 +8573,7 @@
       </c>
       <c r="M43" s="17"/>
       <c r="N43" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O43" s="31">
         <v>0</v>
@@ -8442,10 +8581,9 @@
       <c r="P43" s="31">
         <v>5000000</v>
       </c>
-      <c r="W43" s="66" t="s">
-        <v>242</v>
-      </c>
-      <c r="X43" s="67"/>
+      <c r="W43" s="46" t="s">
+        <v>241</v>
+      </c>
       <c r="Y43" s="47">
         <f>Y40*79/100</f>
         <v>46053050</v>
@@ -8471,8 +8609,8 @@
       <c r="L44" s="4"/>
       <c r="O44" s="36"/>
       <c r="P44" s="36"/>
-      <c r="W44" s="68" t="s">
-        <v>243</v>
+      <c r="W44" s="58" t="s">
+        <v>242</v>
       </c>
       <c r="X44" s="48"/>
       <c r="Y44" s="49">
@@ -9193,7 +9331,7 @@
         <v>412</v>
       </c>
       <c r="M65" s="17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N65" s="17"/>
       <c r="O65" s="31">
@@ -9561,7 +9699,7 @@
       </c>
       <c r="M76" s="17"/>
       <c r="N76" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O76" s="31">
         <v>0</v>
@@ -9597,7 +9735,7 @@
       </c>
       <c r="M77" s="17"/>
       <c r="N77" s="17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O77" s="31">
         <v>0</v>
@@ -9703,7 +9841,7 @@
       </c>
       <c r="M84" s="17"/>
       <c r="N84" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="O84" s="31">
         <v>0</v>
@@ -9721,7 +9859,7 @@
       </c>
       <c r="M85" s="17"/>
       <c r="N85" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="O85" s="31">
         <v>0</v>
@@ -9731,12 +9869,12 @@
       </c>
     </row>
     <row r="86" spans="11:16" x14ac:dyDescent="0.3">
-      <c r="K86" s="59" t="s">
-        <v>198</v>
-      </c>
-      <c r="L86" s="59"/>
-      <c r="M86" s="59"/>
-      <c r="N86" s="59"/>
+      <c r="K86" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="L86" s="60"/>
+      <c r="M86" s="60"/>
+      <c r="N86" s="60"/>
       <c r="O86" s="31">
         <f>SUM(O2:O85)</f>
         <v>1939705000</v>
@@ -9824,13 +9962,13 @@
         <v>124</v>
       </c>
       <c r="N1" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="O1" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="18" t="s">
         <v>211</v>
-      </c>
-      <c r="P1" s="18" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -10063,6 +10201,15 @@
       <c r="J7" s="17" t="s">
         <v>181</v>
       </c>
+      <c r="M7" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="N7" t="s">
+        <v>209</v>
+      </c>
+      <c r="O7" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="17">
@@ -10095,6 +10242,15 @@
       <c r="J8" s="17" t="s">
         <v>181</v>
       </c>
+      <c r="M8" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="N8" s="70">
+        <v>29</v>
+      </c>
+      <c r="O8" s="1">
+        <v>377000000</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="17">
@@ -10127,6 +10283,15 @@
       <c r="J9" s="17" t="s">
         <v>181</v>
       </c>
+      <c r="M9" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="N9" s="70">
+        <v>15</v>
+      </c>
+      <c r="O9" s="1">
+        <v>210000000</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="17">
@@ -10159,6 +10324,15 @@
       <c r="J10" s="17" t="s">
         <v>185</v>
       </c>
+      <c r="M10" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="N10" s="70">
+        <v>10</v>
+      </c>
+      <c r="O10" s="1">
+        <v>160000000</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="17">
@@ -10190,6 +10364,15 @@
       </c>
       <c r="J11" s="17" t="s">
         <v>178</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="N11" s="70">
+        <v>54</v>
+      </c>
+      <c r="O11" s="1">
+        <v>747000000</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">

</xml_diff>